<commit_message>
Default to 2-hour IEX purchase, buy RTM / sell GDAM, BESS ₹0.98 Cr/MWh
The app now opens on P7 2-hour, IEX-purchase charging with T-GNA, buying
on RTM and selling on GDAM, with BESS capex ₹0.98 Cr/MWh. Excel defaults
and the reference results are updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BESS_IEX_Financial_Model.xlsx
+++ b/BESS_IEX_Financial_Model.xlsx
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Own solar</t>
+          <t>IEX + T-GNA</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>DAM</t>
+          <t>RTM</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>DAM</t>
+          <t>GDAM</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="B27" s="22" t="n">
-        <v>1.05</v>
+        <v>0.98</v>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
@@ -77662,7 +77662,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Static values for checking the live sheets. Defaults: solar ₹2.05 Cr/MWp, BESS ₹1.05 Cr/MWh, T-GNA ₹586/MWh, equity-funded cost on unless shown.</t>
+          <t>Static values for checking the live sheets. Defaults: solar ₹2.05 Cr/MWp, BESS ₹0.98 Cr/MWh, IEX cases buy RTM / sell GDAM, T-GNA ₹586/MWh, equity-funded cost on unless shown.</t>
         </is>
       </c>
     </row>
@@ -77768,19 +77768,19 @@
         </is>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.1021016324646834</v>
+        <v>0.1093680481969365</v>
       </c>
       <c r="G5" s="29" t="n">
-        <v>0.1335263917417019</v>
+        <v>0.1498360853883663</v>
       </c>
       <c r="H5" s="34" t="n">
-        <v>81.67226664224044</v>
+        <v>133.3949824798688</v>
       </c>
       <c r="I5" s="34" t="n">
-        <v>1029.026238651734</v>
+        <v>978.4572088376869</v>
       </c>
       <c r="J5" s="46" t="n">
-        <v>1.241520561034958</v>
+        <v>1.295151923487879</v>
       </c>
       <c r="K5" s="26" t="n">
         <v>722.414711629237</v>
@@ -77792,10 +77792,10 @@
         <v>206203.0600555201</v>
       </c>
       <c r="N5" s="34" t="n">
-        <v>156.3447343908438</v>
+        <v>156.597579539914</v>
       </c>
       <c r="O5" s="47" t="n">
-        <v>6.070340926694137</v>
+        <v>5.76561916076859</v>
       </c>
     </row>
     <row r="6">
@@ -77823,19 +77823,19 @@
         </is>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.0986570063979112</v>
+        <v>0.1056490339695396</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>0.1247919668118028</v>
+        <v>0.1397133532442713</v>
       </c>
       <c r="H6" s="34" t="n">
-        <v>55.40819277594968</v>
+        <v>107.1309086135778</v>
       </c>
       <c r="I6" s="34" t="n">
-        <v>1029.026238651734</v>
+        <v>978.4572088376869</v>
       </c>
       <c r="J6" s="46" t="n">
-        <v>1.284748869174804</v>
+        <v>1.340614374913083</v>
       </c>
       <c r="K6" s="26" t="n">
         <v>722.414711629237</v>
@@ -77847,10 +77847,10 @@
         <v>206203.0600555201</v>
       </c>
       <c r="N6" s="34" t="n">
-        <v>136.3447343908438</v>
+        <v>136.597579539914</v>
       </c>
       <c r="O6" s="47" t="n">
-        <v>6.257206046581393</v>
+        <v>5.952484280655846</v>
       </c>
     </row>
     <row r="7">
@@ -77878,19 +77878,19 @@
         </is>
       </c>
       <c r="F7" s="29" t="n">
-        <v>0.1068879665439159</v>
+        <v>0.1143211381341082</v>
       </c>
       <c r="G7" s="29" t="n">
-        <v>0.1442032464566633</v>
+        <v>0.1613132858727243</v>
       </c>
       <c r="H7" s="34" t="n">
-        <v>120.1788199375524</v>
+        <v>171.9015357751806</v>
       </c>
       <c r="I7" s="34" t="n">
-        <v>1029.026238651734</v>
+        <v>978.4572088376869</v>
       </c>
       <c r="J7" s="46" t="n">
-        <v>1.27674948699933</v>
+        <v>1.332201565362276</v>
       </c>
       <c r="K7" s="26" t="n">
         <v>722.414711629237</v>
@@ -77902,10 +77902,10 @@
         <v>206203.0600555201</v>
       </c>
       <c r="N7" s="34" t="n">
-        <v>161.8271080268826</v>
+        <v>162.0799531759528</v>
       </c>
       <c r="O7" s="47" t="n">
-        <v>6.070340926694137</v>
+        <v>5.76561916076859</v>
       </c>
     </row>
     <row r="8">
@@ -77933,19 +77933,19 @@
         </is>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.1033811071538989</v>
+        <v>0.1105336522058397</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>0.1348699714512652</v>
+        <v>0.1505023511354625</v>
       </c>
       <c r="H8" s="34" t="n">
-        <v>93.91474607126153</v>
+        <v>145.6374619088898</v>
       </c>
       <c r="I8" s="34" t="n">
-        <v>1029.026238651734</v>
+        <v>978.4572088376869</v>
       </c>
       <c r="J8" s="46" t="n">
-        <v>1.319977795139176</v>
+        <v>1.37766401678748</v>
       </c>
       <c r="K8" s="26" t="n">
         <v>722.414711629237</v>
@@ -77957,10 +77957,10 @@
         <v>206203.0600555201</v>
       </c>
       <c r="N8" s="34" t="n">
-        <v>141.8271080268826</v>
+        <v>142.0799531759528</v>
       </c>
       <c r="O8" s="47" t="n">
-        <v>6.257206046581393</v>
+        <v>5.952484280655846</v>
       </c>
     </row>
     <row r="9">
@@ -77988,19 +77988,19 @@
         </is>
       </c>
       <c r="F9" s="29" t="n">
-        <v>0.07020734973414811</v>
+        <v>0.09465127953225727</v>
       </c>
       <c r="G9" s="29" t="n">
-        <v>0.06903248905494286</v>
+        <v>0.1173995733168</v>
       </c>
       <c r="H9" s="34" t="n">
-        <v>-120.5384467713661</v>
+        <v>15.59613189200577</v>
       </c>
       <c r="I9" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J9" s="46" t="n">
-        <v>1.041369032836184</v>
+        <v>1.216789954825456</v>
       </c>
       <c r="K9" s="26" t="n">
         <v>722.414711629237</v>
@@ -78012,10 +78012,10 @@
         <v>216810</v>
       </c>
       <c r="N9" s="34" t="n">
-        <v>92.28751190469816</v>
+        <v>104.9167944017982</v>
       </c>
       <c r="O9" s="47" t="n">
-        <v>7.081723927363265</v>
+        <v>6.958620356247659</v>
       </c>
     </row>
     <row r="10">
@@ -78043,19 +78043,19 @@
         </is>
       </c>
       <c r="F10" s="29" t="n">
-        <v>0.06612851901256411</v>
+        <v>0.08983497276431651</v>
       </c>
       <c r="G10" s="29" t="n">
-        <v>0.06097117431811017</v>
+        <v>0.106234299588149</v>
       </c>
       <c r="H10" s="34" t="n">
-        <v>-146.802520637657</v>
+        <v>-10.66794197428507</v>
       </c>
       <c r="I10" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J10" s="46" t="n">
-        <v>1.075099185637211</v>
+        <v>1.263426774446076</v>
       </c>
       <c r="K10" s="26" t="n">
         <v>722.414711629237</v>
@@ -78067,10 +78067,10 @@
         <v>216810</v>
       </c>
       <c r="N10" s="34" t="n">
-        <v>72.28751190469816</v>
+        <v>84.91679440179819</v>
       </c>
       <c r="O10" s="47" t="n">
-        <v>7.26126336636151</v>
+        <v>7.138159795245905</v>
       </c>
     </row>
     <row r="11">
@@ -78098,19 +78098,19 @@
         </is>
       </c>
       <c r="F11" s="29" t="n">
-        <v>0.07760642406661378</v>
+        <v>0.1020639098541539</v>
       </c>
       <c r="G11" s="29" t="n">
-        <v>0.08296206977769194</v>
+        <v>0.1334834718169694</v>
       </c>
       <c r="H11" s="34" t="n">
-        <v>-80.02545817172395</v>
+        <v>56.10912049164809</v>
       </c>
       <c r="I11" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J11" s="46" t="n">
-        <v>1.093149717154253</v>
+        <v>1.272269259451959</v>
       </c>
       <c r="K11" s="26" t="n">
         <v>722.414711629237</v>
@@ -78122,10 +78122,10 @@
         <v>216810</v>
       </c>
       <c r="N11" s="34" t="n">
-        <v>98.22751190469818</v>
+        <v>110.8567944017982</v>
       </c>
       <c r="O11" s="47" t="n">
-        <v>7.081723927363265</v>
+        <v>6.958620356247659</v>
       </c>
     </row>
     <row r="12">
@@ -78153,19 +78153,19 @@
         </is>
       </c>
       <c r="F12" s="29" t="n">
-        <v>0.07340196864476678</v>
+        <v>0.09710513598403125</v>
       </c>
       <c r="G12" s="29" t="n">
-        <v>0.07466880101792095</v>
+        <v>0.1210283596648117</v>
       </c>
       <c r="H12" s="34" t="n">
-        <v>-106.2895320380147</v>
+        <v>29.84504662535722</v>
       </c>
       <c r="I12" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J12" s="46" t="n">
-        <v>1.133330676873366</v>
+        <v>1.321802924184234</v>
       </c>
       <c r="K12" s="26" t="n">
         <v>722.414711629237</v>
@@ -78177,10 +78177,10 @@
         <v>216810</v>
       </c>
       <c r="N12" s="34" t="n">
-        <v>78.22751190469818</v>
+        <v>90.8567944017982</v>
       </c>
       <c r="O12" s="47" t="n">
-        <v>7.26126336636151</v>
+        <v>7.138159795245905</v>
       </c>
     </row>
     <row r="13">
@@ -78218,13 +78218,13 @@
         </is>
       </c>
       <c r="H13" s="34" t="n">
-        <v>-1237.508940980623</v>
+        <v>-1068.679447660996</v>
       </c>
       <c r="I13" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J13" s="46" t="n">
-        <v>-1.129945485290474</v>
+        <v>-0.9766532516227588</v>
       </c>
       <c r="K13" s="26" t="n">
         <v>722.414711629237</v>
@@ -78236,10 +78236,10 @@
         <v>216810</v>
       </c>
       <c r="N13" s="34" t="n">
-        <v>-35.27366793142907</v>
+        <v>-22.64438543432904</v>
       </c>
       <c r="O13" s="47" t="n">
-        <v>13.45189096578642</v>
+        <v>13.32878739467082</v>
       </c>
     </row>
     <row r="14">
@@ -78277,13 +78277,13 @@
         </is>
       </c>
       <c r="H14" s="34" t="n">
-        <v>-1272.607262330738</v>
+        <v>-1103.77776901111</v>
       </c>
       <c r="I14" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J14" s="46" t="n">
-        <v>-1.129945485290474</v>
+        <v>-0.9766532516227588</v>
       </c>
       <c r="K14" s="26" t="n">
         <v>722.414711629237</v>
@@ -78295,10 +78295,10 @@
         <v>216810</v>
       </c>
       <c r="N14" s="34" t="n">
-        <v>-55.27366793142907</v>
+        <v>-42.64438543432904</v>
       </c>
       <c r="O14" s="47" t="n">
-        <v>13.63143040478467</v>
+        <v>13.50832683366906</v>
       </c>
     </row>
     <row r="15">
@@ -78336,13 +78336,13 @@
         </is>
       </c>
       <c r="H15" s="34" t="n">
-        <v>-1183.949798177575</v>
+        <v>-1015.120304857947</v>
       </c>
       <c r="I15" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J15" s="46" t="n">
-        <v>-1.028563174928095</v>
+        <v>-0.8680293476630669</v>
       </c>
       <c r="K15" s="26" t="n">
         <v>722.414711629237</v>
@@ -78354,10 +78354,10 @@
         <v>216810</v>
       </c>
       <c r="N15" s="34" t="n">
-        <v>-29.33366793142908</v>
+        <v>-16.70438543432904</v>
       </c>
       <c r="O15" s="47" t="n">
-        <v>13.45189096578642</v>
+        <v>13.32878739467082</v>
       </c>
     </row>
     <row r="16">
@@ -78395,13 +78395,13 @@
         </is>
       </c>
       <c r="H16" s="34" t="n">
-        <v>-1219.048119527689</v>
+        <v>-1050.218626208062</v>
       </c>
       <c r="I16" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J16" s="46" t="n">
-        <v>-1.028563174928095</v>
+        <v>-0.8680293476630669</v>
       </c>
       <c r="K16" s="26" t="n">
         <v>722.414711629237</v>
@@ -78413,10 +78413,10 @@
         <v>216810</v>
       </c>
       <c r="N16" s="34" t="n">
-        <v>-49.33366793142908</v>
+        <v>-36.70438543432904</v>
       </c>
       <c r="O16" s="47" t="n">
-        <v>13.63143040478467</v>
+        <v>13.50832683366906</v>
       </c>
     </row>
     <row r="17">
@@ -78444,19 +78444,19 @@
         </is>
       </c>
       <c r="F17" s="29" t="n">
-        <v>0.0994157889356112</v>
+        <v>0.1065902928370895</v>
       </c>
       <c r="G17" s="29" t="n">
-        <v>0.1276566118933059</v>
+        <v>0.1435309891211368</v>
       </c>
       <c r="H17" s="34" t="n">
-        <v>120.5017595221596</v>
+        <v>223.947191197416</v>
       </c>
       <c r="I17" s="34" t="n">
-        <v>2058.052477303467</v>
+        <v>1956.914417675374</v>
       </c>
       <c r="J17" s="46" t="n">
-        <v>1.222138915151433</v>
+        <v>1.274768587372348</v>
       </c>
       <c r="K17" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78468,10 +78468,10 @@
         <v>412182.3963456863</v>
       </c>
       <c r="N17" s="34" t="n">
-        <v>306.6570723059999</v>
+        <v>307.1627626041403</v>
       </c>
       <c r="O17" s="47" t="n">
-        <v>6.076454013365136</v>
+        <v>5.771562897547593</v>
       </c>
     </row>
     <row r="18">
@@ -78499,19 +78499,19 @@
         </is>
       </c>
       <c r="F18" s="29" t="n">
-        <v>0.09769608949070607</v>
+        <v>0.1047332350370506</v>
       </c>
       <c r="G18" s="29" t="n">
-        <v>0.1233442032245403</v>
+        <v>0.138523538574164</v>
       </c>
       <c r="H18" s="34" t="n">
-        <v>94.23768565586916</v>
+        <v>197.6831173311255</v>
       </c>
       <c r="I18" s="34" t="n">
-        <v>2058.052477303467</v>
+        <v>1956.914417675374</v>
       </c>
       <c r="J18" s="46" t="n">
-        <v>1.243753069221357</v>
+        <v>1.29749981308495</v>
       </c>
       <c r="K18" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78523,10 +78523,10 @@
         <v>412182.3963456863</v>
       </c>
       <c r="N18" s="34" t="n">
-        <v>286.6570723059999</v>
+        <v>287.1627626041403</v>
       </c>
       <c r="O18" s="47" t="n">
-        <v>6.169938498690224</v>
+        <v>5.865047382872683</v>
       </c>
     </row>
     <row r="19">
@@ -78554,19 +78554,19 @@
         </is>
       </c>
       <c r="F19" s="29" t="n">
-        <v>0.1042303803215195</v>
+        <v>0.1115709172812068</v>
       </c>
       <c r="G19" s="29" t="n">
-        <v>0.1382450712972761</v>
+        <v>0.1549099880262875</v>
       </c>
       <c r="H19" s="34" t="n">
-        <v>197.4838069571461</v>
+        <v>300.9292386324029</v>
       </c>
       <c r="I19" s="34" t="n">
-        <v>2058.052477303467</v>
+        <v>1956.914417675374</v>
       </c>
       <c r="J19" s="46" t="n">
-        <v>1.257350730512008</v>
+        <v>1.31180023432565</v>
       </c>
       <c r="K19" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78578,10 +78578,10 @@
         <v>412182.3963456863</v>
       </c>
       <c r="N19" s="34" t="n">
-        <v>317.6164940269519</v>
+        <v>318.1221843250923</v>
       </c>
       <c r="O19" s="47" t="n">
-        <v>6.076454013365136</v>
+        <v>5.771562897547593</v>
       </c>
     </row>
     <row r="20">
@@ -78609,19 +78609,19 @@
         </is>
       </c>
       <c r="F20" s="29" t="n">
-        <v>0.1024793156517884</v>
+        <v>0.1096793432514663</v>
       </c>
       <c r="G20" s="29" t="n">
-        <v>0.1336295299523439</v>
+        <v>0.1495529957024045</v>
       </c>
       <c r="H20" s="34" t="n">
-        <v>171.2197330908554</v>
+        <v>274.6651647661123</v>
       </c>
       <c r="I20" s="34" t="n">
-        <v>2058.052477303467</v>
+        <v>1956.914417675374</v>
       </c>
       <c r="J20" s="46" t="n">
-        <v>1.278964884581931</v>
+        <v>1.334531460038252</v>
       </c>
       <c r="K20" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78633,10 +78633,10 @@
         <v>412182.3963456863</v>
       </c>
       <c r="N20" s="34" t="n">
-        <v>297.6164940269519</v>
+        <v>298.1221843250923</v>
       </c>
       <c r="O20" s="47" t="n">
-        <v>6.169938498690224</v>
+        <v>5.865047382872683</v>
       </c>
     </row>
     <row r="21">
@@ -78664,19 +78664,19 @@
         </is>
       </c>
       <c r="F21" s="29" t="n">
-        <v>0.06141877272429752</v>
+        <v>0.08482042809196744</v>
       </c>
       <c r="G21" s="29" t="n">
-        <v>0.05320304276460985</v>
+        <v>0.09712023502651579</v>
       </c>
       <c r="H21" s="34" t="n">
-        <v>-334.7489390101846</v>
+        <v>-73.98927177895145</v>
       </c>
       <c r="I21" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J21" s="46" t="n">
-        <v>0.9815067172747397</v>
+        <v>1.14477109551286</v>
       </c>
       <c r="K21" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78688,10 +78688,10 @@
         <v>433620</v>
       </c>
       <c r="N21" s="34" t="n">
-        <v>170.8408617712599</v>
+        <v>194.4119094153343</v>
       </c>
       <c r="O21" s="47" t="n">
-        <v>7.217079200139809</v>
+        <v>7.154936256419749</v>
       </c>
     </row>
     <row r="22">
@@ -78719,19 +78719,19 @@
         </is>
       </c>
       <c r="F22" s="29" t="n">
-        <v>0.05942881851937887</v>
+        <v>0.08247565809426283</v>
       </c>
       <c r="G22" s="29" t="n">
-        <v>0.04951191039143865</v>
+        <v>0.09214223624441453</v>
       </c>
       <c r="H22" s="34" t="n">
-        <v>-361.0130128764757</v>
+        <v>-100.2533456452424</v>
       </c>
       <c r="I22" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J22" s="46" t="n">
-        <v>0.9951014366575985</v>
+        <v>1.176187178419729</v>
       </c>
       <c r="K22" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78743,10 +78743,10 @@
         <v>433620</v>
       </c>
       <c r="N22" s="34" t="n">
-        <v>150.8408617712599</v>
+        <v>174.4119094153343</v>
       </c>
       <c r="O22" s="47" t="n">
-        <v>7.306848919638932</v>
+        <v>7.244705975918872</v>
       </c>
     </row>
     <row r="23">
@@ -78774,19 +78774,19 @@
         </is>
       </c>
       <c r="F23" s="29" t="n">
-        <v>0.06904457119723284</v>
+        <v>0.09241559282980927</v>
       </c>
       <c r="G23" s="29" t="n">
-        <v>0.06689501204920301</v>
+        <v>0.1126842449061477</v>
       </c>
       <c r="H23" s="34" t="n">
-        <v>-253.6343396483383</v>
+        <v>7.036705420332783</v>
       </c>
       <c r="I23" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J23" s="46" t="n">
-        <v>1.033344036716282</v>
+        <v>1.200250400139363</v>
       </c>
       <c r="K23" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78798,10 +78798,10 @@
         <v>433620</v>
       </c>
       <c r="N23" s="34" t="n">
-        <v>182.7338555212599</v>
+        <v>206.2919094153343</v>
       </c>
       <c r="O23" s="47" t="n">
-        <v>7.217079200139809</v>
+        <v>7.154936256419749</v>
       </c>
     </row>
     <row r="24">
@@ -78829,19 +78829,19 @@
         </is>
       </c>
       <c r="F24" s="29" t="n">
-        <v>0.06699071200887652</v>
+        <v>0.08999850263673526</v>
       </c>
       <c r="G24" s="29" t="n">
-        <v>0.06325787910610237</v>
+        <v>0.1070903367676442</v>
       </c>
       <c r="H24" s="34" t="n">
-        <v>-279.898413514629</v>
+        <v>-19.22736844595777</v>
       </c>
       <c r="I24" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J24" s="46" t="n">
-        <v>1.062665714096026</v>
+        <v>1.231666483046231</v>
       </c>
       <c r="K24" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78853,10 +78853,10 @@
         <v>433620</v>
       </c>
       <c r="N24" s="34" t="n">
-        <v>162.7338555212599</v>
+        <v>186.2919094153343</v>
       </c>
       <c r="O24" s="47" t="n">
-        <v>7.306848919638932</v>
+        <v>7.244705975918872</v>
       </c>
     </row>
     <row r="25">
@@ -78884,19 +78884,19 @@
         </is>
       </c>
       <c r="F25" s="29" t="n">
-        <v>-0.06569098135453083</v>
+        <v>-0.01755575398728776</v>
       </c>
       <c r="G25" s="29" t="n">
-        <v>-0.1459720535062012</v>
+        <v>-0.07731771702833362</v>
       </c>
       <c r="H25" s="34" t="n">
-        <v>-1218.305346561501</v>
+        <v>-920.5304691312272</v>
       </c>
       <c r="I25" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J25" s="46" t="n">
-        <v>0.2120192076320566</v>
+        <v>0.44573637177076</v>
       </c>
       <c r="K25" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78908,10 +78908,10 @@
         <v>433620</v>
       </c>
       <c r="N25" s="34" t="n">
-        <v>58.27850209900537</v>
+        <v>81.84954974307985</v>
       </c>
       <c r="O25" s="47" t="n">
-        <v>10.05626492487989</v>
+        <v>9.994121981159832</v>
       </c>
     </row>
     <row r="26">
@@ -78939,19 +78939,19 @@
         </is>
       </c>
       <c r="F26" s="29" t="n">
-        <v>-0.06741131264881089</v>
+        <v>-0.01916609190354707</v>
       </c>
       <c r="G26" s="29" t="n">
-        <v>-0.1465317452451576</v>
+        <v>-0.07855729893996838</v>
       </c>
       <c r="H26" s="34" t="n">
-        <v>-1253.403667911616</v>
+        <v>-946.7945429975182</v>
       </c>
       <c r="I26" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J26" s="46" t="n">
-        <v>0.2120192076320566</v>
+        <v>0.44573637177076</v>
       </c>
       <c r="K26" s="26" t="n">
         <v>1444.829423258474</v>
@@ -78963,10 +78963,10 @@
         <v>433620</v>
       </c>
       <c r="N26" s="34" t="n">
-        <v>38.27850209900537</v>
+        <v>61.84954974307984</v>
       </c>
       <c r="O26" s="47" t="n">
-        <v>10.14603464437902</v>
+        <v>10.08389170065895</v>
       </c>
     </row>
     <row r="27">
@@ -78994,19 +78994,19 @@
         </is>
       </c>
       <c r="F27" s="29" t="n">
-        <v>-0.04142817723216147</v>
+        <v>-0.003318224646259693</v>
       </c>
       <c r="G27" s="29" t="n">
-        <v>-0.111812901331248</v>
+        <v>-0.05603398279427124</v>
       </c>
       <c r="H27" s="34" t="n">
-        <v>-1115.662857435046</v>
+        <v>-835.148866742452</v>
       </c>
       <c r="I27" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J27" s="46" t="n">
-        <v>0.3135124048963943</v>
+        <v>0.5543602757304519</v>
       </c>
       <c r="K27" s="26" t="n">
         <v>1444.829423258474</v>
@@ -79018,10 +79018,10 @@
         <v>433620</v>
       </c>
       <c r="N27" s="34" t="n">
-        <v>70.17149584900537</v>
+        <v>93.72954974307984</v>
       </c>
       <c r="O27" s="47" t="n">
-        <v>10.05626492487989</v>
+        <v>9.994121981159832</v>
       </c>
     </row>
     <row r="28">
@@ -79049,19 +79049,19 @@
         </is>
       </c>
       <c r="F28" s="29" t="n">
-        <v>-0.04310549605033315</v>
+        <v>-0.005004959852649316</v>
       </c>
       <c r="G28" s="29" t="n">
-        <v>-0.1126177028430531</v>
+        <v>-0.05757952931804994</v>
       </c>
       <c r="H28" s="34" t="n">
-        <v>-1147.321103873838</v>
+        <v>-861.4129406087427</v>
       </c>
       <c r="I28" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J28" s="46" t="n">
-        <v>0.3135124048963943</v>
+        <v>0.5543602757304519</v>
       </c>
       <c r="K28" s="26" t="n">
         <v>1444.829423258474</v>
@@ -79073,10 +79073,10 @@
         <v>433620</v>
       </c>
       <c r="N28" s="34" t="n">
-        <v>50.17149584900537</v>
+        <v>73.72954974307984</v>
       </c>
       <c r="O28" s="47" t="n">
-        <v>10.14603464437902</v>
+        <v>10.08389170065895</v>
       </c>
     </row>
     <row r="29">
@@ -79104,19 +79104,19 @@
         </is>
       </c>
       <c r="F29" s="29" t="n">
-        <v>0.1000126600657772</v>
+        <v>0.1070823536469293</v>
       </c>
       <c r="G29" s="29" t="n">
-        <v>0.1289128071501481</v>
+        <v>0.1445849172968098</v>
       </c>
       <c r="H29" s="34" t="n">
-        <v>66.10304326631258</v>
+        <v>117.8257591039409</v>
       </c>
       <c r="I29" s="34" t="n">
-        <v>1045.810870101535</v>
+        <v>995.2418402874886</v>
       </c>
       <c r="J29" s="46" t="n">
-        <v>1.22525530769098</v>
+        <v>1.277155733335908</v>
       </c>
       <c r="K29" s="26" t="n">
         <v>722.414711629237</v>
@@ -79128,10 +79128,10 @@
         <v>206203.0600555208</v>
       </c>
       <c r="N29" s="34" t="n">
-        <v>156.3223932130559</v>
+        <v>156.5752383621261</v>
       </c>
       <c r="O29" s="47" t="n">
-        <v>6.162220585095212</v>
+        <v>5.857498819169668</v>
       </c>
     </row>
     <row r="30">
@@ -79159,19 +79159,19 @@
         </is>
       </c>
       <c r="F30" s="29" t="n">
-        <v>0.09665101775153973</v>
+        <v>0.1034581428218005</v>
       </c>
       <c r="G30" s="29" t="n">
-        <v>0.1205735909293512</v>
+        <v>0.1349435484246507</v>
       </c>
       <c r="H30" s="34" t="n">
-        <v>39.83896940002174</v>
+        <v>91.56168523765004</v>
       </c>
       <c r="I30" s="34" t="n">
-        <v>1045.810870101535</v>
+        <v>995.2418402874886</v>
       </c>
       <c r="J30" s="46" t="n">
-        <v>1.267789827650698</v>
+        <v>1.321851466099288</v>
       </c>
       <c r="K30" s="26" t="n">
         <v>722.414711629237</v>
@@ -79183,10 +79183,10 @@
         <v>206203.0600555208</v>
       </c>
       <c r="N30" s="34" t="n">
-        <v>136.3223932130559</v>
+        <v>136.5752383621261</v>
       </c>
       <c r="O30" s="47" t="n">
-        <v>6.349085704982468</v>
+        <v>6.044363939056923</v>
       </c>
     </row>
     <row r="31">
@@ -79214,19 +79214,19 @@
         </is>
       </c>
       <c r="F31" s="29" t="n">
-        <v>0.1047425445817441</v>
+        <v>0.1119728825483713</v>
       </c>
       <c r="G31" s="29" t="n">
-        <v>0.1393374879798027</v>
+        <v>0.1557744241783457</v>
       </c>
       <c r="H31" s="34" t="n">
-        <v>104.6095965616243</v>
+        <v>156.3323123992527</v>
       </c>
       <c r="I31" s="34" t="n">
-        <v>1045.810870101535</v>
+        <v>995.2418402874886</v>
       </c>
       <c r="J31" s="46" t="n">
-        <v>1.259918830717221</v>
+        <v>1.313580537548708</v>
       </c>
       <c r="K31" s="26" t="n">
         <v>722.414711629237</v>
@@ -79238,10 +79238,10 @@
         <v>206203.0600555208</v>
       </c>
       <c r="N31" s="34" t="n">
-        <v>161.8047668490947</v>
+        <v>162.0576119981649</v>
       </c>
       <c r="O31" s="47" t="n">
-        <v>6.162220585095212</v>
+        <v>5.857498819169668</v>
       </c>
     </row>
     <row r="32">
@@ -79269,19 +79269,19 @@
         </is>
       </c>
       <c r="F32" s="29" t="n">
-        <v>0.1013206271446426</v>
+        <v>0.1082824521043971</v>
       </c>
       <c r="G32" s="29" t="n">
-        <v>0.1304275815874271</v>
+        <v>0.1454768960379677</v>
       </c>
       <c r="H32" s="34" t="n">
-        <v>78.34552269533336</v>
+        <v>130.0682385329619</v>
       </c>
       <c r="I32" s="34" t="n">
-        <v>1045.810870101535</v>
+        <v>995.2418402874886</v>
       </c>
       <c r="J32" s="46" t="n">
-        <v>1.30245335067694</v>
+        <v>1.358276270312088</v>
       </c>
       <c r="K32" s="26" t="n">
         <v>722.414711629237</v>
@@ -79293,10 +79293,10 @@
         <v>206203.0600555208</v>
       </c>
       <c r="N32" s="34" t="n">
-        <v>141.8047668490947</v>
+        <v>142.0576119981649</v>
       </c>
       <c r="O32" s="47" t="n">
-        <v>6.349085704982468</v>
+        <v>6.044363939056923</v>
       </c>
     </row>
     <row r="33">
@@ -79324,19 +79324,19 @@
         </is>
       </c>
       <c r="F33" s="29" t="n">
-        <v>0.07020734973414811</v>
+        <v>0.09465127953225727</v>
       </c>
       <c r="G33" s="29" t="n">
-        <v>0.06903248905494286</v>
+        <v>0.1173995733168</v>
       </c>
       <c r="H33" s="34" t="n">
-        <v>-120.5384467713661</v>
+        <v>15.59613189200577</v>
       </c>
       <c r="I33" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J33" s="46" t="n">
-        <v>1.041369032836184</v>
+        <v>1.216789954825456</v>
       </c>
       <c r="K33" s="26" t="n">
         <v>722.414711629237</v>
@@ -79348,10 +79348,10 @@
         <v>216810</v>
       </c>
       <c r="N33" s="34" t="n">
-        <v>92.28751190469816</v>
+        <v>104.9167944017982</v>
       </c>
       <c r="O33" s="47" t="n">
-        <v>7.081723927363265</v>
+        <v>6.958620356247659</v>
       </c>
     </row>
     <row r="34">
@@ -79379,19 +79379,19 @@
         </is>
       </c>
       <c r="F34" s="29" t="n">
-        <v>0.06612851901256411</v>
+        <v>0.08983497276431651</v>
       </c>
       <c r="G34" s="29" t="n">
-        <v>0.06097117431811017</v>
+        <v>0.106234299588149</v>
       </c>
       <c r="H34" s="34" t="n">
-        <v>-146.802520637657</v>
+        <v>-10.66794197428507</v>
       </c>
       <c r="I34" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J34" s="46" t="n">
-        <v>1.075099185637211</v>
+        <v>1.263426774446076</v>
       </c>
       <c r="K34" s="26" t="n">
         <v>722.414711629237</v>
@@ -79403,10 +79403,10 @@
         <v>216810</v>
       </c>
       <c r="N34" s="34" t="n">
-        <v>72.28751190469816</v>
+        <v>84.91679440179819</v>
       </c>
       <c r="O34" s="47" t="n">
-        <v>7.26126336636151</v>
+        <v>7.138159795245905</v>
       </c>
     </row>
     <row r="35">
@@ -79434,19 +79434,19 @@
         </is>
       </c>
       <c r="F35" s="29" t="n">
-        <v>0.07760642406661378</v>
+        <v>0.1020639098541539</v>
       </c>
       <c r="G35" s="29" t="n">
-        <v>0.08296206977769194</v>
+        <v>0.1334834718169694</v>
       </c>
       <c r="H35" s="34" t="n">
-        <v>-80.02545817172395</v>
+        <v>56.10912049164809</v>
       </c>
       <c r="I35" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J35" s="46" t="n">
-        <v>1.093149717154253</v>
+        <v>1.272269259451959</v>
       </c>
       <c r="K35" s="26" t="n">
         <v>722.414711629237</v>
@@ -79458,10 +79458,10 @@
         <v>216810</v>
       </c>
       <c r="N35" s="34" t="n">
-        <v>98.22751190469818</v>
+        <v>110.8567944017982</v>
       </c>
       <c r="O35" s="47" t="n">
-        <v>7.081723927363265</v>
+        <v>6.958620356247659</v>
       </c>
     </row>
     <row r="36">
@@ -79489,19 +79489,19 @@
         </is>
       </c>
       <c r="F36" s="29" t="n">
-        <v>0.07340196864476678</v>
+        <v>0.09710513598403125</v>
       </c>
       <c r="G36" s="29" t="n">
-        <v>0.07466880101792095</v>
+        <v>0.1210283596648117</v>
       </c>
       <c r="H36" s="34" t="n">
-        <v>-106.2895320380147</v>
+        <v>29.84504662535722</v>
       </c>
       <c r="I36" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J36" s="46" t="n">
-        <v>1.133330676873366</v>
+        <v>1.321802924184234</v>
       </c>
       <c r="K36" s="26" t="n">
         <v>722.414711629237</v>
@@ -79513,10 +79513,10 @@
         <v>216810</v>
       </c>
       <c r="N36" s="34" t="n">
-        <v>78.22751190469818</v>
+        <v>90.8567944017982</v>
       </c>
       <c r="O36" s="47" t="n">
-        <v>7.26126336636151</v>
+        <v>7.138159795245905</v>
       </c>
     </row>
     <row r="37">
@@ -79554,13 +79554,13 @@
         </is>
       </c>
       <c r="H37" s="34" t="n">
-        <v>-1237.508940980623</v>
+        <v>-1068.679447660996</v>
       </c>
       <c r="I37" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J37" s="46" t="n">
-        <v>-1.129945485290474</v>
+        <v>-0.9766532516227588</v>
       </c>
       <c r="K37" s="26" t="n">
         <v>722.414711629237</v>
@@ -79572,10 +79572,10 @@
         <v>216810</v>
       </c>
       <c r="N37" s="34" t="n">
-        <v>-35.27366793142907</v>
+        <v>-22.64438543432904</v>
       </c>
       <c r="O37" s="47" t="n">
-        <v>13.45189096578642</v>
+        <v>13.32878739467082</v>
       </c>
     </row>
     <row r="38">
@@ -79613,13 +79613,13 @@
         </is>
       </c>
       <c r="H38" s="34" t="n">
-        <v>-1272.607262330738</v>
+        <v>-1103.77776901111</v>
       </c>
       <c r="I38" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J38" s="46" t="n">
-        <v>-1.129945485290474</v>
+        <v>-0.9766532516227588</v>
       </c>
       <c r="K38" s="26" t="n">
         <v>722.414711629237</v>
@@ -79631,10 +79631,10 @@
         <v>216810</v>
       </c>
       <c r="N38" s="34" t="n">
-        <v>-55.27366793142907</v>
+        <v>-42.64438543432904</v>
       </c>
       <c r="O38" s="47" t="n">
-        <v>13.63143040478467</v>
+        <v>13.50832683366906</v>
       </c>
     </row>
     <row r="39">
@@ -79672,13 +79672,13 @@
         </is>
       </c>
       <c r="H39" s="34" t="n">
-        <v>-1183.949798177575</v>
+        <v>-1015.120304857947</v>
       </c>
       <c r="I39" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J39" s="46" t="n">
-        <v>-1.028563174928095</v>
+        <v>-0.8680293476630669</v>
       </c>
       <c r="K39" s="26" t="n">
         <v>722.414711629237</v>
@@ -79690,10 +79690,10 @@
         <v>216810</v>
       </c>
       <c r="N39" s="34" t="n">
-        <v>-29.33366793142908</v>
+        <v>-16.70438543432904</v>
       </c>
       <c r="O39" s="47" t="n">
-        <v>13.45189096578642</v>
+        <v>13.32878739467082</v>
       </c>
     </row>
     <row r="40">
@@ -79731,13 +79731,13 @@
         </is>
       </c>
       <c r="H40" s="34" t="n">
-        <v>-1219.048119527689</v>
+        <v>-1050.218626208062</v>
       </c>
       <c r="I40" s="34" t="n">
-        <v>758.5354472106989</v>
+        <v>707.9664173966522</v>
       </c>
       <c r="J40" s="46" t="n">
-        <v>-1.028563174928095</v>
+        <v>-0.8680293476630669</v>
       </c>
       <c r="K40" s="26" t="n">
         <v>722.414711629237</v>
@@ -79749,10 +79749,10 @@
         <v>216810</v>
       </c>
       <c r="N40" s="34" t="n">
-        <v>-49.33366793142908</v>
+        <v>-36.70438543432904</v>
       </c>
       <c r="O40" s="47" t="n">
-        <v>13.63143040478467</v>
+        <v>13.50832683366906</v>
       </c>
     </row>
     <row r="41">
@@ -79780,19 +79780,19 @@
         </is>
       </c>
       <c r="F41" s="29" t="n">
-        <v>0.09729769827278811</v>
+        <v>0.1042768396531309</v>
       </c>
       <c r="G41" s="29" t="n">
-        <v>0.123050472386747</v>
+        <v>0.1382977356521028</v>
       </c>
       <c r="H41" s="34" t="n">
-        <v>88.39201287657666</v>
+        <v>191.8374445518334</v>
       </c>
       <c r="I41" s="34" t="n">
-        <v>2091.621740203071</v>
+        <v>1990.483680574977</v>
       </c>
       <c r="J41" s="46" t="n">
-        <v>1.20575120035253</v>
+        <v>1.25666060678427</v>
       </c>
       <c r="K41" s="26" t="n">
         <v>1444.829423258474</v>
@@ -79804,10 +79804,10 @@
         <v>412073.6562798821</v>
       </c>
       <c r="N41" s="34" t="n">
-        <v>306.4752575074364</v>
+        <v>306.9809478055768</v>
       </c>
       <c r="O41" s="47" t="n">
-        <v>6.171178860129384</v>
+        <v>5.866203696826856</v>
       </c>
     </row>
     <row r="42">
@@ -79835,19 +79835,19 @@
         </is>
       </c>
       <c r="F42" s="29" t="n">
-        <v>0.09561989743765198</v>
+        <v>0.1024676508136882</v>
       </c>
       <c r="G42" s="29" t="n">
-        <v>0.1189387284810765</v>
+        <v>0.1335353421545132</v>
       </c>
       <c r="H42" s="34" t="n">
-        <v>62.1279390102864</v>
+        <v>165.5733706855426</v>
       </c>
       <c r="I42" s="34" t="n">
-        <v>2091.621740203071</v>
+        <v>1990.483680574977</v>
       </c>
       <c r="J42" s="46" t="n">
-        <v>1.227018460332389</v>
+        <v>1.27900847316596</v>
       </c>
       <c r="K42" s="26" t="n">
         <v>1444.829423258474</v>
@@ -79859,10 +79859,10 @@
         <v>412073.6562798821</v>
       </c>
       <c r="N42" s="34" t="n">
-        <v>286.4752575074364</v>
+        <v>286.9809478055768</v>
       </c>
       <c r="O42" s="47" t="n">
-        <v>6.264689115755637</v>
+        <v>5.959713952453108</v>
       </c>
     </row>
     <row r="43">
@@ -79890,19 +79890,19 @@
         </is>
       </c>
       <c r="F43" s="29" t="n">
-        <v>0.1020564342692237</v>
+        <v>0.1091955042558893</v>
       </c>
       <c r="G43" s="29" t="n">
-        <v>0.1333881965636877</v>
+        <v>0.1493898875229999</v>
       </c>
       <c r="H43" s="34" t="n">
-        <v>165.3709232924516</v>
+        <v>268.8163549677082</v>
       </c>
       <c r="I43" s="34" t="n">
-        <v>2091.621740203071</v>
+        <v>1990.483680574977</v>
       </c>
       <c r="J43" s="46" t="n">
-        <v>1.24039618693086</v>
+        <v>1.29306593269749</v>
       </c>
       <c r="K43" s="26" t="n">
         <v>1444.829423258474</v>
@@ -79914,10 +79914,10 @@
         <v>412073.6562798821</v>
       </c>
       <c r="N43" s="34" t="n">
-        <v>317.4341413401133</v>
+        <v>317.9398316382537</v>
       </c>
       <c r="O43" s="47" t="n">
-        <v>6.171178860129384</v>
+        <v>5.866203696826856</v>
       </c>
     </row>
     <row r="44">
@@ -79945,19 +79945,19 @@
         </is>
       </c>
       <c r="F44" s="29" t="n">
-        <v>0.1003482584550964</v>
+        <v>0.1073529383444488</v>
       </c>
       <c r="G44" s="29" t="n">
-        <v>0.1289880169624887</v>
+        <v>0.1442947478170754</v>
       </c>
       <c r="H44" s="34" t="n">
-        <v>139.1068494261605</v>
+        <v>242.5522811014175</v>
       </c>
       <c r="I44" s="34" t="n">
-        <v>2091.621740203071</v>
+        <v>1990.483680574977</v>
       </c>
       <c r="J44" s="46" t="n">
-        <v>1.261663446910719</v>
+        <v>1.31541379907918</v>
       </c>
       <c r="K44" s="26" t="n">
         <v>1444.829423258474</v>
@@ -79969,10 +79969,10 @@
         <v>412073.6562798821</v>
       </c>
       <c r="N44" s="34" t="n">
-        <v>297.4341413401133</v>
+        <v>297.9398316382537</v>
       </c>
       <c r="O44" s="47" t="n">
-        <v>6.264689115755637</v>
+        <v>5.959713952453108</v>
       </c>
     </row>
     <row r="45">
@@ -80000,19 +80000,19 @@
         </is>
       </c>
       <c r="F45" s="29" t="n">
-        <v>0.06141877272429752</v>
+        <v>0.08482042809196744</v>
       </c>
       <c r="G45" s="29" t="n">
-        <v>0.05320304276460985</v>
+        <v>0.09712023502651579</v>
       </c>
       <c r="H45" s="34" t="n">
-        <v>-334.7489390101846</v>
+        <v>-73.98927177895145</v>
       </c>
       <c r="I45" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J45" s="46" t="n">
-        <v>0.9815067172747397</v>
+        <v>1.14477109551286</v>
       </c>
       <c r="K45" s="26" t="n">
         <v>1444.829423258474</v>
@@ -80024,10 +80024,10 @@
         <v>433620</v>
       </c>
       <c r="N45" s="34" t="n">
-        <v>170.8408617712599</v>
+        <v>194.4119094153343</v>
       </c>
       <c r="O45" s="47" t="n">
-        <v>7.217079200139809</v>
+        <v>7.154936256419749</v>
       </c>
     </row>
     <row r="46">
@@ -80055,19 +80055,19 @@
         </is>
       </c>
       <c r="F46" s="29" t="n">
-        <v>0.05942881851937887</v>
+        <v>0.08247565809426283</v>
       </c>
       <c r="G46" s="29" t="n">
-        <v>0.04951191039143865</v>
+        <v>0.09214223624441453</v>
       </c>
       <c r="H46" s="34" t="n">
-        <v>-361.0130128764757</v>
+        <v>-100.2533456452424</v>
       </c>
       <c r="I46" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J46" s="46" t="n">
-        <v>0.9951014366575985</v>
+        <v>1.176187178419729</v>
       </c>
       <c r="K46" s="26" t="n">
         <v>1444.829423258474</v>
@@ -80079,10 +80079,10 @@
         <v>433620</v>
       </c>
       <c r="N46" s="34" t="n">
-        <v>150.8408617712599</v>
+        <v>174.4119094153343</v>
       </c>
       <c r="O46" s="47" t="n">
-        <v>7.306848919638932</v>
+        <v>7.244705975918872</v>
       </c>
     </row>
     <row r="47">
@@ -80110,19 +80110,19 @@
         </is>
       </c>
       <c r="F47" s="29" t="n">
-        <v>0.06904457119723284</v>
+        <v>0.09241559282980927</v>
       </c>
       <c r="G47" s="29" t="n">
-        <v>0.06689501204920301</v>
+        <v>0.1126842449061477</v>
       </c>
       <c r="H47" s="34" t="n">
-        <v>-253.6343396483383</v>
+        <v>7.036705420332783</v>
       </c>
       <c r="I47" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J47" s="46" t="n">
-        <v>1.033344036716282</v>
+        <v>1.200250400139363</v>
       </c>
       <c r="K47" s="26" t="n">
         <v>1444.829423258474</v>
@@ -80134,10 +80134,10 @@
         <v>433620</v>
       </c>
       <c r="N47" s="34" t="n">
-        <v>182.7338555212599</v>
+        <v>206.2919094153343</v>
       </c>
       <c r="O47" s="47" t="n">
-        <v>7.217079200139809</v>
+        <v>7.154936256419749</v>
       </c>
     </row>
     <row r="48">
@@ -80165,19 +80165,19 @@
         </is>
       </c>
       <c r="F48" s="29" t="n">
-        <v>0.06699071200887652</v>
+        <v>0.08999850263673526</v>
       </c>
       <c r="G48" s="29" t="n">
-        <v>0.06325787910610237</v>
+        <v>0.1070903367676442</v>
       </c>
       <c r="H48" s="34" t="n">
-        <v>-279.898413514629</v>
+        <v>-19.22736844595777</v>
       </c>
       <c r="I48" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J48" s="46" t="n">
-        <v>1.062665714096026</v>
+        <v>1.231666483046231</v>
       </c>
       <c r="K48" s="26" t="n">
         <v>1444.829423258474</v>
@@ -80189,10 +80189,10 @@
         <v>433620</v>
       </c>
       <c r="N48" s="34" t="n">
-        <v>162.7338555212599</v>
+        <v>186.2919094153343</v>
       </c>
       <c r="O48" s="47" t="n">
-        <v>7.306848919638932</v>
+        <v>7.244705975918872</v>
       </c>
     </row>
     <row r="49">
@@ -80220,19 +80220,19 @@
         </is>
       </c>
       <c r="F49" s="29" t="n">
-        <v>-0.06569098135453083</v>
+        <v>-0.01755575398728776</v>
       </c>
       <c r="G49" s="29" t="n">
-        <v>-0.1459720535062012</v>
+        <v>-0.07731771702833362</v>
       </c>
       <c r="H49" s="34" t="n">
-        <v>-1218.305346561501</v>
+        <v>-920.5304691312272</v>
       </c>
       <c r="I49" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J49" s="46" t="n">
-        <v>0.2120192076320566</v>
+        <v>0.44573637177076</v>
       </c>
       <c r="K49" s="26" t="n">
         <v>1444.829423258474</v>
@@ -80244,10 +80244,10 @@
         <v>433620</v>
       </c>
       <c r="N49" s="34" t="n">
-        <v>58.27850209900537</v>
+        <v>81.84954974307985</v>
       </c>
       <c r="O49" s="47" t="n">
-        <v>10.05626492487989</v>
+        <v>9.994121981159832</v>
       </c>
     </row>
     <row r="50">
@@ -80275,19 +80275,19 @@
         </is>
       </c>
       <c r="F50" s="29" t="n">
-        <v>-0.06741131264881089</v>
+        <v>-0.01916609190354707</v>
       </c>
       <c r="G50" s="29" t="n">
-        <v>-0.1465317452451576</v>
+        <v>-0.07855729893996838</v>
       </c>
       <c r="H50" s="34" t="n">
-        <v>-1253.403667911616</v>
+        <v>-946.7945429975182</v>
       </c>
       <c r="I50" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J50" s="46" t="n">
-        <v>0.2120192076320566</v>
+        <v>0.44573637177076</v>
       </c>
       <c r="K50" s="26" t="n">
         <v>1444.829423258474</v>
@@ -80299,10 +80299,10 @@
         <v>433620</v>
       </c>
       <c r="N50" s="34" t="n">
-        <v>38.27850209900537</v>
+        <v>61.84954974307984</v>
       </c>
       <c r="O50" s="47" t="n">
-        <v>10.14603464437902</v>
+        <v>10.08389170065895</v>
       </c>
     </row>
     <row r="51">
@@ -80330,19 +80330,19 @@
         </is>
       </c>
       <c r="F51" s="29" t="n">
-        <v>-0.04142817723216147</v>
+        <v>-0.003318224646259693</v>
       </c>
       <c r="G51" s="29" t="n">
-        <v>-0.111812901331248</v>
+        <v>-0.05603398279427124</v>
       </c>
       <c r="H51" s="34" t="n">
-        <v>-1115.662857435046</v>
+        <v>-835.148866742452</v>
       </c>
       <c r="I51" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J51" s="46" t="n">
-        <v>0.3135124048963943</v>
+        <v>0.5543602757304519</v>
       </c>
       <c r="K51" s="26" t="n">
         <v>1444.829423258474</v>
@@ -80354,10 +80354,10 @@
         <v>433620</v>
       </c>
       <c r="N51" s="34" t="n">
-        <v>70.17149584900537</v>
+        <v>93.72954974307984</v>
       </c>
       <c r="O51" s="47" t="n">
-        <v>10.05626492487989</v>
+        <v>9.994121981159832</v>
       </c>
     </row>
     <row r="52">
@@ -80385,19 +80385,19 @@
         </is>
       </c>
       <c r="F52" s="29" t="n">
-        <v>-0.04310549605033315</v>
+        <v>-0.005004959852649316</v>
       </c>
       <c r="G52" s="29" t="n">
-        <v>-0.1126177028430531</v>
+        <v>-0.05757952931804994</v>
       </c>
       <c r="H52" s="34" t="n">
-        <v>-1147.321103873838</v>
+        <v>-861.4129406087427</v>
       </c>
       <c r="I52" s="34" t="n">
-        <v>1517.070894421398</v>
+        <v>1415.932834793304</v>
       </c>
       <c r="J52" s="46" t="n">
-        <v>0.3135124048963943</v>
+        <v>0.5543602757304519</v>
       </c>
       <c r="K52" s="26" t="n">
         <v>1444.829423258474</v>
@@ -80409,10 +80409,10 @@
         <v>433620</v>
       </c>
       <c r="N52" s="34" t="n">
-        <v>50.17149584900537</v>
+        <v>73.72954974307984</v>
       </c>
       <c r="O52" s="47" t="n">
-        <v>10.14603464437902</v>
+        <v>10.08389170065895</v>
       </c>
     </row>
     <row r="53">
@@ -80440,19 +80440,19 @@
         </is>
       </c>
       <c r="F53" s="29" t="n">
-        <v>0.1000196590226471</v>
+        <v>0.1070886570351205</v>
       </c>
       <c r="G53" s="29" t="n">
-        <v>0.1289277500757063</v>
+        <v>0.1445986130078097</v>
       </c>
       <c r="H53" s="34" t="n">
-        <v>55.13998975407381</v>
+        <v>98.24225295209723</v>
       </c>
       <c r="I53" s="34" t="n">
-        <v>871.6166522092909</v>
+        <v>829.4757940309186</v>
       </c>
       <c r="J53" s="46" t="n">
-        <v>1.225201556021121</v>
+        <v>1.277092518695436</v>
       </c>
       <c r="K53" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80464,10 +80464,10 @@
         <v>171835.8833796001</v>
       </c>
       <c r="N53" s="34" t="n">
-        <v>130.2776582407759</v>
+        <v>130.4883625316678</v>
       </c>
       <c r="O53" s="47" t="n">
-        <v>6.161643427194505</v>
+        <v>5.856921661268959</v>
       </c>
     </row>
     <row r="54">
@@ -80495,19 +80495,19 @@
         </is>
       </c>
       <c r="F54" s="29" t="n">
-        <v>0.09599956062532844</v>
+        <v>0.1027552524194454</v>
       </c>
       <c r="G54" s="29" t="n">
-        <v>0.1190177034288605</v>
+        <v>0.1331489492321466</v>
       </c>
       <c r="H54" s="34" t="n">
-        <v>28.87591588778295</v>
+        <v>71.97817908580626</v>
       </c>
       <c r="I54" s="34" t="n">
-        <v>871.6166522092909</v>
+        <v>829.4757940309186</v>
       </c>
       <c r="J54" s="46" t="n">
-        <v>1.276236679335565</v>
+        <v>1.330720440870542</v>
       </c>
       <c r="K54" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80519,10 +80519,10 @@
         <v>171835.8833796001</v>
       </c>
       <c r="N54" s="34" t="n">
-        <v>110.2776582407759</v>
+        <v>110.4883625316678</v>
       </c>
       <c r="O54" s="47" t="n">
-        <v>6.385881571059213</v>
+        <v>6.081159805133669</v>
       </c>
     </row>
     <row r="55">
@@ -80550,19 +80550,19 @@
         </is>
       </c>
       <c r="F55" s="29" t="n">
-        <v>0.1047488723162421</v>
+        <v>0.1119784694473652</v>
       </c>
       <c r="G55" s="29" t="n">
-        <v>0.139351177373526</v>
+        <v>0.1557866098915383</v>
       </c>
       <c r="H55" s="34" t="n">
-        <v>87.22878416683305</v>
+        <v>130.3310473648567</v>
       </c>
       <c r="I55" s="34" t="n">
-        <v>871.6166522092909</v>
+        <v>829.4757940309186</v>
       </c>
       <c r="J55" s="46" t="n">
-        <v>1.259860800125137</v>
+        <v>1.313512598137707</v>
       </c>
       <c r="K55" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80574,10 +80574,10 @@
         <v>171835.8833796001</v>
       </c>
       <c r="N55" s="34" t="n">
-        <v>134.8463029374747</v>
+        <v>135.0570072283665</v>
       </c>
       <c r="O55" s="47" t="n">
-        <v>6.161643427194505</v>
+        <v>5.856921661268959</v>
       </c>
     </row>
     <row r="56">
@@ -80605,19 +80605,19 @@
         </is>
       </c>
       <c r="F56" s="29" t="n">
-        <v>0.1006566656428199</v>
+        <v>0.107565850313775</v>
       </c>
       <c r="G56" s="29" t="n">
-        <v>0.1287645516707506</v>
+        <v>0.1435590998808197</v>
       </c>
       <c r="H56" s="34" t="n">
-        <v>60.96471030054229</v>
+        <v>104.0669734985658</v>
       </c>
       <c r="I56" s="34" t="n">
-        <v>871.6166522092909</v>
+        <v>829.4757940309186</v>
       </c>
       <c r="J56" s="46" t="n">
-        <v>1.310895923439582</v>
+        <v>1.367140520312813</v>
       </c>
       <c r="K56" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80629,10 +80629,10 @@
         <v>171835.8833796001</v>
       </c>
       <c r="N56" s="34" t="n">
-        <v>114.8463029374747</v>
+        <v>115.0570072283665</v>
       </c>
       <c r="O56" s="47" t="n">
-        <v>6.385881571059213</v>
+        <v>6.081159805133669</v>
       </c>
     </row>
     <row r="57">
@@ -80660,19 +80660,19 @@
         </is>
       </c>
       <c r="F57" s="29" t="n">
-        <v>0.07020734973414811</v>
+        <v>0.09465127953225727</v>
       </c>
       <c r="G57" s="29" t="n">
-        <v>0.06903248905494286</v>
+        <v>0.1173995733167997</v>
       </c>
       <c r="H57" s="34" t="n">
-        <v>-100.4487056428053</v>
+        <v>12.99677657667115</v>
       </c>
       <c r="I57" s="34" t="n">
-        <v>632.1128726755824</v>
+        <v>589.9720144972101</v>
       </c>
       <c r="J57" s="46" t="n">
-        <v>1.041369032836183</v>
+        <v>1.216789954825456</v>
       </c>
       <c r="K57" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80684,10 +80684,10 @@
         <v>180675</v>
       </c>
       <c r="N57" s="34" t="n">
-        <v>76.90625992058179</v>
+        <v>87.43066200149846</v>
       </c>
       <c r="O57" s="47" t="n">
-        <v>7.081723927363267</v>
+        <v>6.958620356247666</v>
       </c>
     </row>
     <row r="58">
@@ -80715,19 +80715,19 @@
         </is>
       </c>
       <c r="F58" s="29" t="n">
-        <v>0.06533570275495448</v>
+        <v>0.08890045090367715</v>
       </c>
       <c r="G58" s="29" t="n">
-        <v>0.05920885504396567</v>
+        <v>0.1041866260693337</v>
       </c>
       <c r="H58" s="34" t="n">
-        <v>-126.7127795090961</v>
+        <v>-13.26729728961966</v>
       </c>
       <c r="I58" s="34" t="n">
-        <v>632.1128726755824</v>
+        <v>589.9720144972101</v>
       </c>
       <c r="J58" s="46" t="n">
-        <v>1.075099185637211</v>
+        <v>1.263426774446076</v>
       </c>
       <c r="K58" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80739,10 +80739,10 @@
         <v>180675</v>
       </c>
       <c r="N58" s="34" t="n">
-        <v>56.9062599205818</v>
+        <v>67.43066200149846</v>
       </c>
       <c r="O58" s="47" t="n">
-        <v>7.297171254161163</v>
+        <v>7.174067683045562</v>
       </c>
     </row>
     <row r="59">
@@ -80770,19 +80770,19 @@
         </is>
       </c>
       <c r="F59" s="29" t="n">
-        <v>0.07760642406661378</v>
+        <v>0.1020639098541539</v>
       </c>
       <c r="G59" s="29" t="n">
-        <v>0.08296206977769194</v>
+        <v>0.1334834718169694</v>
       </c>
       <c r="H59" s="34" t="n">
-        <v>-66.68788180977009</v>
+        <v>46.75760040970655</v>
       </c>
       <c r="I59" s="34" t="n">
-        <v>632.1128726755824</v>
+        <v>589.9720144972101</v>
       </c>
       <c r="J59" s="46" t="n">
-        <v>1.093149717154252</v>
+        <v>1.272269259451959</v>
       </c>
       <c r="K59" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80794,10 +80794,10 @@
         <v>180675</v>
       </c>
       <c r="N59" s="34" t="n">
-        <v>81.85625992058179</v>
+        <v>92.38066200149846</v>
       </c>
       <c r="O59" s="47" t="n">
-        <v>7.081723927363267</v>
+        <v>6.958620356247666</v>
       </c>
     </row>
     <row r="60">
@@ -80825,19 +80825,19 @@
         </is>
       </c>
       <c r="F60" s="29" t="n">
-        <v>0.07258469000414436</v>
+        <v>0.09614286065962252</v>
       </c>
       <c r="G60" s="29" t="n">
-        <v>0.07267881365591922</v>
+        <v>0.1187504947005954</v>
       </c>
       <c r="H60" s="34" t="n">
-        <v>-92.95195567606081</v>
+        <v>20.49352654341574</v>
       </c>
       <c r="I60" s="34" t="n">
-        <v>632.1128726755824</v>
+        <v>589.9720144972101</v>
       </c>
       <c r="J60" s="46" t="n">
-        <v>1.133330676873366</v>
+        <v>1.321802924184233</v>
       </c>
       <c r="K60" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80849,10 +80849,10 @@
         <v>180675</v>
       </c>
       <c r="N60" s="34" t="n">
-        <v>61.85625992058179</v>
+        <v>72.38066200149846</v>
       </c>
       <c r="O60" s="47" t="n">
-        <v>7.297171254161163</v>
+        <v>7.174067683045562</v>
       </c>
     </row>
     <row r="61">
@@ -80890,13 +80890,13 @@
         </is>
       </c>
       <c r="H61" s="34" t="n">
-        <v>-1031.257450817186</v>
+        <v>-890.5662063841633</v>
       </c>
       <c r="I61" s="34" t="n">
-        <v>632.1128726755824</v>
+        <v>589.9720144972101</v>
       </c>
       <c r="J61" s="46" t="n">
-        <v>-1.129945485290475</v>
+        <v>-0.9766532516227604</v>
       </c>
       <c r="K61" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80908,10 +80908,10 @@
         <v>180675</v>
       </c>
       <c r="N61" s="34" t="n">
-        <v>-29.39472327619091</v>
+        <v>-18.87032119527425</v>
       </c>
       <c r="O61" s="47" t="n">
-        <v>13.45189096578643</v>
+        <v>13.32878739467082</v>
       </c>
     </row>
     <row r="62">
@@ -80949,13 +80949,13 @@
         </is>
       </c>
       <c r="H62" s="34" t="n">
-        <v>-1066.355772167301</v>
+        <v>-925.664527734278</v>
       </c>
       <c r="I62" s="34" t="n">
-        <v>632.1128726755824</v>
+        <v>589.9720144972101</v>
       </c>
       <c r="J62" s="46" t="n">
-        <v>-1.129945485290475</v>
+        <v>-0.9766532516227604</v>
       </c>
       <c r="K62" s="26" t="n">
         <v>602.0122596910307</v>
@@ -80967,10 +80967,10 @@
         <v>180675</v>
       </c>
       <c r="N62" s="34" t="n">
-        <v>-49.39472327619091</v>
+        <v>-38.87032119527424</v>
       </c>
       <c r="O62" s="47" t="n">
-        <v>13.66733829258433</v>
+        <v>13.54423472146872</v>
       </c>
     </row>
     <row r="63">
@@ -81008,13 +81008,13 @@
         </is>
       </c>
       <c r="H63" s="34" t="n">
-        <v>-986.6248318146457</v>
+        <v>-845.9335873816229</v>
       </c>
       <c r="I63" s="34" t="n">
-        <v>632.1128726755824</v>
+        <v>589.9720144972101</v>
       </c>
       <c r="J63" s="46" t="n">
-        <v>-1.028563174928096</v>
+        <v>-0.8680293476630679</v>
       </c>
       <c r="K63" s="26" t="n">
         <v>602.0122596910307</v>
@@ -81026,10 +81026,10 @@
         <v>180675</v>
       </c>
       <c r="N63" s="34" t="n">
-        <v>-24.44472327619091</v>
+        <v>-13.92032119527425</v>
       </c>
       <c r="O63" s="47" t="n">
-        <v>13.45189096578643</v>
+        <v>13.32878739467082</v>
       </c>
     </row>
     <row r="64">
@@ -81067,13 +81067,13 @@
         </is>
       </c>
       <c r="H64" s="34" t="n">
-        <v>-1021.723153164761</v>
+        <v>-881.0319087317379</v>
       </c>
       <c r="I64" s="34" t="n">
-        <v>632.1128726755824</v>
+        <v>589.9720144972101</v>
       </c>
       <c r="J64" s="46" t="n">
-        <v>-1.028563174928096</v>
+        <v>-0.8680293476630679</v>
       </c>
       <c r="K64" s="26" t="n">
         <v>602.0122596910307</v>
@@ -81085,10 +81085,10 @@
         <v>180675</v>
       </c>
       <c r="N64" s="34" t="n">
-        <v>-44.44472327619091</v>
+        <v>-33.92032119527425</v>
       </c>
       <c r="O64" s="47" t="n">
-        <v>13.66733829258433</v>
+        <v>13.54423472146872</v>
       </c>
     </row>
     <row r="65">
@@ -81116,19 +81116,19 @@
         </is>
       </c>
       <c r="F65" s="29" t="n">
-        <v>0.09733883211806382</v>
+        <v>0.1043184198125205</v>
       </c>
       <c r="G65" s="29" t="n">
-        <v>0.1231384208076712</v>
+        <v>0.1383897856238111</v>
       </c>
       <c r="H65" s="34" t="n">
-        <v>74.22063424593516</v>
+        <v>160.4251606419824</v>
       </c>
       <c r="I65" s="34" t="n">
-        <v>1743.233304418582</v>
+        <v>1658.951588061837</v>
       </c>
       <c r="J65" s="46" t="n">
-        <v>1.20594219539094</v>
+        <v>1.256854701562048</v>
       </c>
       <c r="K65" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81140,10 +81140,10 @@
         <v>343444.7514706115</v>
       </c>
       <c r="N65" s="34" t="n">
-        <v>255.4779307462588</v>
+        <v>255.8993393280425</v>
       </c>
       <c r="O65" s="47" t="n">
-        <v>6.169034575407149</v>
+        <v>5.864105878490562</v>
       </c>
     </row>
     <row r="66">
@@ -81171,19 +81171,19 @@
         </is>
       </c>
       <c r="F66" s="29" t="n">
-        <v>0.09532881096173662</v>
+        <v>0.1021511767674222</v>
       </c>
       <c r="G66" s="29" t="n">
-        <v>0.118226511759265</v>
+        <v>0.132702752650674</v>
       </c>
       <c r="H66" s="34" t="n">
-        <v>47.95656037964446</v>
+        <v>134.1610867756916</v>
       </c>
       <c r="I66" s="34" t="n">
-        <v>1743.233304418582</v>
+        <v>1658.951588061837</v>
       </c>
       <c r="J66" s="46" t="n">
-        <v>1.231459757048162</v>
+        <v>1.283668662649601</v>
       </c>
       <c r="K66" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81195,10 +81195,10 @@
         <v>343444.7514706115</v>
       </c>
       <c r="N66" s="34" t="n">
-        <v>235.4779307462588</v>
+        <v>235.8993393280425</v>
       </c>
       <c r="O66" s="47" t="n">
-        <v>6.281229785355439</v>
+        <v>5.976301088438849</v>
       </c>
     </row>
     <row r="67">
@@ -81226,19 +81226,19 @@
         </is>
       </c>
       <c r="F67" s="29" t="n">
-        <v>0.1020965958962109</v>
+        <v>0.1092360789716519</v>
       </c>
       <c r="G67" s="29" t="n">
-        <v>0.1334761635069269</v>
+        <v>0.1494818577395175</v>
       </c>
       <c r="H67" s="34" t="n">
-        <v>138.3711105417093</v>
+        <v>224.5756369377563</v>
       </c>
       <c r="I67" s="34" t="n">
-        <v>1743.233304418582</v>
+        <v>1658.951588061837</v>
       </c>
       <c r="J67" s="46" t="n">
-        <v>1.240583805664471</v>
+        <v>1.293256251301097</v>
       </c>
       <c r="K67" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81250,10 +81250,10 @@
         <v>343444.7514706115</v>
       </c>
       <c r="N67" s="34" t="n">
-        <v>264.6105712958508</v>
+        <v>265.0319798776345</v>
       </c>
       <c r="O67" s="47" t="n">
-        <v>6.169034575407149</v>
+        <v>5.864105878490562</v>
       </c>
     </row>
     <row r="68">
@@ -81281,19 +81281,19 @@
         </is>
       </c>
       <c r="F68" s="29" t="n">
-        <v>0.1000501861498221</v>
+        <v>0.1070288525485591</v>
       </c>
       <c r="G68" s="29" t="n">
-        <v>0.1282202445959059</v>
+        <v>0.1433980110580889</v>
       </c>
       <c r="H68" s="34" t="n">
-        <v>112.1070366754183</v>
+        <v>198.3115630714654</v>
       </c>
       <c r="I68" s="34" t="n">
-        <v>1743.233304418582</v>
+        <v>1658.951588061837</v>
       </c>
       <c r="J68" s="46" t="n">
-        <v>1.266101367321693</v>
+        <v>1.32007021238865</v>
       </c>
       <c r="K68" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81305,10 +81305,10 @@
         <v>343444.7514706115</v>
       </c>
       <c r="N68" s="34" t="n">
-        <v>244.6105712958508</v>
+        <v>245.0319798776345</v>
       </c>
       <c r="O68" s="47" t="n">
-        <v>6.281229785355439</v>
+        <v>5.976301088438849</v>
       </c>
     </row>
     <row r="69">
@@ -81336,19 +81336,19 @@
         </is>
       </c>
       <c r="F69" s="29" t="n">
-        <v>0.06141877272429752</v>
+        <v>0.08482042809196744</v>
       </c>
       <c r="G69" s="29" t="n">
-        <v>0.05320304276460985</v>
+        <v>0.09712023502651579</v>
       </c>
       <c r="H69" s="34" t="n">
-        <v>-278.9574491751542</v>
+        <v>-61.65772648245991</v>
       </c>
       <c r="I69" s="34" t="n">
-        <v>1264.225745351165</v>
+        <v>1179.94402899442</v>
       </c>
       <c r="J69" s="46" t="n">
-        <v>0.9815067172747394</v>
+        <v>1.14477109551286</v>
       </c>
       <c r="K69" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81360,10 +81360,10 @@
         <v>361350</v>
       </c>
       <c r="N69" s="34" t="n">
-        <v>142.3673848093832</v>
+        <v>162.0099245127786</v>
       </c>
       <c r="O69" s="47" t="n">
-        <v>7.217079200139813</v>
+        <v>7.154936256419751</v>
       </c>
     </row>
     <row r="70">
@@ -81391,19 +81391,19 @@
         </is>
       </c>
       <c r="F70" s="29" t="n">
-        <v>0.05903651877106764</v>
+        <v>0.08201383200946288</v>
       </c>
       <c r="G70" s="29" t="n">
-        <v>0.04868658856855224</v>
+        <v>0.09118795214568987</v>
       </c>
       <c r="H70" s="34" t="n">
-        <v>-305.221523041445</v>
+        <v>-87.92180034875066</v>
       </c>
       <c r="I70" s="34" t="n">
-        <v>1264.225745351165</v>
+        <v>1179.94402899442</v>
       </c>
       <c r="J70" s="46" t="n">
-        <v>0.9951014366575982</v>
+        <v>1.182470395001102</v>
       </c>
       <c r="K70" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81415,10 +81415,10 @@
         <v>361350</v>
       </c>
       <c r="N70" s="34" t="n">
-        <v>122.3673848093832</v>
+        <v>142.0099245127786</v>
       </c>
       <c r="O70" s="47" t="n">
-        <v>7.324802863538761</v>
+        <v>7.262659919818698</v>
       </c>
     </row>
     <row r="71">
@@ -81446,19 +81446,19 @@
         </is>
       </c>
       <c r="F71" s="29" t="n">
-        <v>0.06904457119723284</v>
+        <v>0.09241559282980927</v>
       </c>
       <c r="G71" s="29" t="n">
-        <v>0.06689501204920278</v>
+        <v>0.1126842449061477</v>
       </c>
       <c r="H71" s="34" t="n">
-        <v>-211.3619497069486</v>
+        <v>5.863921183610597</v>
       </c>
       <c r="I71" s="34" t="n">
-        <v>1264.225745351165</v>
+        <v>1179.94402899442</v>
       </c>
       <c r="J71" s="46" t="n">
-        <v>1.033344036716281</v>
+        <v>1.200250400139363</v>
       </c>
       <c r="K71" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81470,10 +81470,10 @@
         <v>361350</v>
       </c>
       <c r="N71" s="34" t="n">
-        <v>152.2782129343832</v>
+        <v>171.9099245127785</v>
       </c>
       <c r="O71" s="47" t="n">
-        <v>7.217079200139813</v>
+        <v>7.154936256419751</v>
       </c>
     </row>
     <row r="72">
@@ -81501,19 +81501,19 @@
         </is>
       </c>
       <c r="F72" s="29" t="n">
-        <v>0.0665858043085924</v>
+        <v>0.08952240685735957</v>
       </c>
       <c r="G72" s="29" t="n">
-        <v>0.06247024454254679</v>
+        <v>0.1060199045390159</v>
       </c>
       <c r="H72" s="34" t="n">
-        <v>-237.6260235732396</v>
+        <v>-20.40015268268007</v>
       </c>
       <c r="I72" s="34" t="n">
-        <v>1264.225745351165</v>
+        <v>1179.94402899442</v>
       </c>
       <c r="J72" s="46" t="n">
-        <v>1.064374882389981</v>
+        <v>1.237949699627605</v>
       </c>
       <c r="K72" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81525,10 +81525,10 @@
         <v>361350</v>
       </c>
       <c r="N72" s="34" t="n">
-        <v>132.2782129343832</v>
+        <v>151.9099245127785</v>
       </c>
       <c r="O72" s="47" t="n">
-        <v>7.324802863538761</v>
+        <v>7.262659919818698</v>
       </c>
     </row>
     <row r="73">
@@ -81556,19 +81556,19 @@
         </is>
       </c>
       <c r="F73" s="29" t="n">
-        <v>-0.06569098135453094</v>
+        <v>-0.01755575398728787</v>
       </c>
       <c r="G73" s="29" t="n">
-        <v>-0.1459720535062014</v>
+        <v>-0.07731771702833362</v>
       </c>
       <c r="H73" s="34" t="n">
-        <v>-1015.254455467918</v>
+        <v>-767.1087242760226</v>
       </c>
       <c r="I73" s="34" t="n">
-        <v>1264.225745351165</v>
+        <v>1179.94402899442</v>
       </c>
       <c r="J73" s="46" t="n">
-        <v>0.2120192076320557</v>
+        <v>0.44573637177076</v>
       </c>
       <c r="K73" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81580,10 +81580,10 @@
         <v>361350</v>
       </c>
       <c r="N73" s="34" t="n">
-        <v>48.56541841583774</v>
+        <v>68.20795811923313</v>
       </c>
       <c r="O73" s="47" t="n">
-        <v>10.0562649248799</v>
+        <v>9.994121981159843</v>
       </c>
     </row>
     <row r="74">
@@ -81611,19 +81611,19 @@
         </is>
       </c>
       <c r="F74" s="29" t="n">
-        <v>-0.06774880870198291</v>
+        <v>-0.01951673590112929</v>
       </c>
       <c r="G74" s="29" t="n">
-        <v>-0.1466425002979775</v>
+        <v>-0.0788003381460099</v>
       </c>
       <c r="H74" s="34" t="n">
-        <v>-1050.352776818033</v>
+        <v>-793.8125073760009</v>
       </c>
       <c r="I74" s="34" t="n">
-        <v>1264.225745351165</v>
+        <v>1179.94402899442</v>
       </c>
       <c r="J74" s="46" t="n">
-        <v>0.2120192076320557</v>
+        <v>0.44573637177076</v>
       </c>
       <c r="K74" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81635,10 +81635,10 @@
         <v>361350</v>
       </c>
       <c r="N74" s="34" t="n">
-        <v>28.56541841583774</v>
+        <v>48.20795811923313</v>
       </c>
       <c r="O74" s="47" t="n">
-        <v>10.16398858827885</v>
+        <v>10.10184564455879</v>
       </c>
     </row>
     <row r="75">
@@ -81666,19 +81666,19 @@
         </is>
       </c>
       <c r="F75" s="29" t="n">
-        <v>-0.04142817723216158</v>
+        <v>-0.003318224646259804</v>
       </c>
       <c r="G75" s="29" t="n">
-        <v>-0.1118129013312482</v>
+        <v>-0.05603398279427124</v>
       </c>
       <c r="H75" s="34" t="n">
-        <v>-929.7190478625381</v>
+        <v>-695.9573889520436</v>
       </c>
       <c r="I75" s="34" t="n">
-        <v>1264.225745351165</v>
+        <v>1179.94402899442</v>
       </c>
       <c r="J75" s="46" t="n">
-        <v>0.3135124048963939</v>
+        <v>0.5543602757304519</v>
       </c>
       <c r="K75" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81690,10 +81690,10 @@
         <v>361350</v>
       </c>
       <c r="N75" s="34" t="n">
-        <v>58.47624654083774</v>
+        <v>78.10795811923313</v>
       </c>
       <c r="O75" s="47" t="n">
-        <v>10.0562649248799</v>
+        <v>9.994121981159843</v>
       </c>
     </row>
     <row r="76">
@@ -81721,19 +81721,19 @@
         </is>
       </c>
       <c r="F76" s="29" t="n">
-        <v>-0.04347026417533223</v>
+        <v>-0.005337096448255696</v>
       </c>
       <c r="G76" s="29" t="n">
-        <v>-0.1127764082389768</v>
+        <v>-0.05788148683047839</v>
       </c>
       <c r="H76" s="34" t="n">
-        <v>-961.9506401198845</v>
+        <v>-722.2214628183342</v>
       </c>
       <c r="I76" s="34" t="n">
-        <v>1264.225745351165</v>
+        <v>1179.94402899442</v>
       </c>
       <c r="J76" s="46" t="n">
-        <v>0.3135124048963939</v>
+        <v>0.5543602757304519</v>
       </c>
       <c r="K76" s="26" t="n">
         <v>1204.024519382061</v>
@@ -81745,10 +81745,10 @@
         <v>361350</v>
       </c>
       <c r="N76" s="34" t="n">
-        <v>38.47624654083774</v>
+        <v>58.10795811923313</v>
       </c>
       <c r="O76" s="47" t="n">
-        <v>10.16398858827885</v>
+        <v>10.10184564455879</v>
       </c>
     </row>
     <row r="78">

</xml_diff>